<commit_message>
Added connections to H2 and power networks. Run? Yes. Works? Don't know yet
</commit_message>
<xml_diff>
--- a/case_studies/2030/carriers_list.xlsx
+++ b/case_studies/2030/carriers_list.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\case_studies\current_layout_optimal\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\case_studies\2030\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C504E9C-C6B4-4BA6-8253-2196AE4B5A59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E61D0149-FD35-4A4E-8E6A-AD3F9A57FF73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>electricity</t>
   </si>
@@ -94,6 +94,9 @@
   </si>
   <si>
     <t>electricity_grid</t>
+  </si>
+  <si>
+    <t>hydrogen_transported</t>
   </si>
 </sst>
 </file>
@@ -420,7 +423,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
@@ -538,6 +541,11 @@
         <v>22</v>
       </c>
     </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
new model for cracker and decommissioning
</commit_message>
<xml_diff>
--- a/case_studies/2030/carriers_list.xlsx
+++ b/case_studies/2030/carriers_list.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\case_studies\2030\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\case_studies\current_layout\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1FE2263-154A-49B2-B16A-EA87B491E95E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BB15016-E36B-4378-9C6F-FF3AC2E08AF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>electricity</t>
   </si>
@@ -97,6 +97,9 @@
   </si>
   <si>
     <t>hydrogen_transported</t>
+  </si>
+  <si>
+    <t>cracking_byproducts</t>
   </si>
 </sst>
 </file>
@@ -423,7 +426,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
@@ -546,6 +549,11 @@
         <v>23</v>
       </c>
     </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>24</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>